<commit_message>
Update monthly plan: ₹1.2L Zerodha, Pluxee ₹5,600 groceries, no CC
- Investment target raised to ₹120,000/month
- Pluxee benefit (₹4,400 + ₹1,200) covers groceries; ₹0 from salary
- New Monthly Plan sheet with step-by-step salary allocation
- Projected salary surplus ~₹8,653 after all targets

Co-authored-by: Shivam Modnaval <ShivamModanval5268@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget-tracker/monthly_budget_tracker.xlsx
+++ b/budget-tracker/monthly_budget_tracker.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Transaction Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="June 2026 Baseline" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Monthly Plan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,9 +21,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,6 +41,10 @@
     <font>
       <b val="1"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -73,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -82,8 +87,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,13 +456,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -508,7 +515,7 @@
         <v>71000</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>55000</v>
+        <v>120000</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>0</v>
@@ -523,7 +530,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Fixed monthly SIP; adjust based on liquidity needs</t>
+          <t>Transfer ₹1.2L to Zerodha on 1st–2nd of month</t>
         </is>
       </c>
     </row>
@@ -537,7 +544,7 @@
         <v>18060</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>18060</v>
+        <v>18000</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -566,7 +573,7 @@
         <v>13180</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>0</v>
@@ -581,21 +588,21 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Audit CC statement monthly; pay via UPI when possible</t>
+          <t>No CC bills — pay everything via UPI/debit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Groceries</t>
+          <t>Pluxee — groceries (benefit)</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>2178</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>2000</v>
+        <v>5600</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0</v>
@@ -610,21 +617,21 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>DMart/BigBasket bulk orders</t>
+          <t>₹4,400 + ₹1,200 loaded monthly; DMart/BigBasket only</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Restaurant dining</t>
+          <t>Groceries (from salary)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>5253</v>
+        <v>2178</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
@@ -639,18 +646,18 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Max 2–3 sit-down meals per month</t>
+          <t>Use Pluxee first; salary only if Pluxee exhausted</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Street food / canteen</t>
+          <t>Restaurant dining</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>3594</v>
+        <v>5253</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>2500</v>
@@ -668,21 +675,21 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Office lunch alternatives</t>
+          <t>Max 2 sit-down meals per month</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Desserts (Polar Bear etc.)</t>
+          <t>Street food / canteen</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>924</v>
+        <v>3594</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>300</v>
+        <v>2500</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
@@ -697,18 +704,18 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Max 1–2 visits per month</t>
+          <t>Office lunch — use Infosys cafeteria when possible</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Office snacks / tea</t>
+          <t>Desserts (Polar Bear etc.)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>750</v>
+        <v>924</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>300</v>
@@ -726,21 +733,21 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Carry flask; use Infosys cafeteria</t>
+          <t>Max 1 visit per month</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Office cafe (Cowrks)</t>
+          <t>Office snacks / tea</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>598</v>
+        <v>750</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0</v>
@@ -755,18 +762,18 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Use only when necessary</t>
+          <t>Carry flask; avoid daily ₹35 UPI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Transport (Metro)</t>
+          <t>Office cafe (Cowrks)</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>180</v>
+        <v>598</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>200</v>
@@ -784,21 +791,21 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Already optimal</t>
+          <t>Use only when necessary</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Software subscriptions</t>
+          <t>Transport (Metro)</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>2376</v>
+        <v>180</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0</v>
@@ -813,21 +820,21 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Cursor AI — review tier / annual plan</t>
+          <t>Already optimal</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Other subscriptions</t>
+          <t>Software subscriptions</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2</v>
+        <v>2376</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0</v>
@@ -842,21 +849,21 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>YouTube, streaming, etc.</t>
+          <t>Cursor AI — review tier / annual plan</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Other subscriptions</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2290</v>
+        <v>2</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2500</v>
+        <v>200</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -871,21 +878,21 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Variable; claim via corporate insurance</t>
+          <t>YouTube, streaming, etc.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Education / training</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>1875</v>
+        <v>2290</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
@@ -900,21 +907,21 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Skill-building — keep if ROI-positive</t>
+          <t>Variable; claim via corporate insurance</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Shopping (Amazon etc.)</t>
+          <t>Education / training</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>1842</v>
+        <v>1875</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0</v>
@@ -929,21 +936,21 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Non-gift discretionary purchases</t>
+          <t>Only if actively enrolled in a course</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Gift cards</t>
+          <t>Shopping (Amazon etc.)</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>4240</v>
+        <v>1842</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0</v>
@@ -958,21 +965,21 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Avoid prepaid unless planned gift</t>
+          <t>Non-essential purchases only</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Luxury / big purchases</t>
+          <t>Gift cards</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>30867</v>
+        <v>4240</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
@@ -987,21 +994,21 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Sinking fund: max ₹2,500/month accrual</t>
+          <t>Avoid prepaid unless planned gift</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Misc / buffer</t>
+          <t>Luxury / big purchases</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>0</v>
+        <v>30867</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0</v>
@@ -1016,63 +1023,122 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Unexpected expenses</t>
+          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Misc / buffer</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <f>D20-C20</f>
+        <v/>
+      </c>
+      <c r="F20" s="2">
+        <f>IF(D20=0,"Enter spend",IF(E20&lt;=0,"✓ On track","⚠ Over"))</f>
+        <v/>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Unexpected expenses from salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>TOTAL (excl. income)</t>
         </is>
       </c>
-      <c r="B20" s="5">
-        <f>SUM(B2:B19)</f>
-        <v/>
-      </c>
-      <c r="C20" s="5">
-        <f>SUM(C2:C19)</f>
-        <v/>
-      </c>
-      <c r="D20" s="5">
-        <f>SUM(D2:D19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="5">
-        <f>D20-C20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Monthly salary (target income)</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>158853</v>
-      </c>
-    </row>
+      <c r="B21" s="5">
+        <f>SUM(B2:B20)</f>
+        <v/>
+      </c>
+      <c r="C21" s="5">
+        <f>SUM(C2:C20)</f>
+        <v/>
+      </c>
+      <c r="D21" s="5">
+        <f>SUM(D2:D20)</f>
+        <v/>
+      </c>
+      <c r="E21" s="5">
+        <f>D21-C21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Projected surplus (Income − Actual spend)</t>
-        </is>
-      </c>
-      <c r="D23" s="5">
-        <f>C22-D20</f>
-        <v/>
+          <t>Monthly salary (bank)</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>158853</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Savings rate (%)</t>
-        </is>
-      </c>
-      <c r="D24" s="6">
-        <f>IF(C22&gt;0,D23/C22,0)</f>
+          <t>Pluxee grocery benefit (separate)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Zerodha investment target</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Living spend from salary (target)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>30200</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Projected salary surplus (Salary − Actual spend)</t>
+        </is>
+      </c>
+      <c r="D27" s="5">
+        <f>C23-D21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Total to Zerodha + surplus wealth</t>
+        </is>
+      </c>
+      <c r="C28" s="5">
+        <f>C25+C27</f>
         <v/>
       </c>
     </row>
@@ -1439,7 +1505,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Investments (Zerodha),Family transfers,Credit card payment,Groceries,Restaurant dining,Street food / canteen,Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Misc / buffer"</formula1>
+      <formula1>"Investments (Zerodha),Family transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Restaurant dining,Street food / canteen,Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Debit,Credit"</formula1>
@@ -1903,17 +1969,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
-        <is>
-          <t>Monthly Budget Dashboard</t>
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Monthly Budget Dashboard — Updated Plan</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1990,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Key targets (based on June 2026 analysis)</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -1932,7 +1998,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Monthly salary</t>
+          <t>Monthly salary (bank)</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
@@ -1942,96 +2008,617 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Target living expenses</t>
+          <t>Pluxee groceries (₹4,400 + ₹1,200)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>53113</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Target investments</t>
+          <t>Total monthly resources</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>55000</v>
+        <v>164453</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Target family transfers</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n">
-        <v>18060</v>
-      </c>
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Target projected surplus</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>32780</v>
-      </c>
+          <t>Fixed outflows (from salary)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
-      <c r="B9" t="inlineStr"/>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Zerodha investment</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>120000</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rules of thumb</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
+          <t>Family transfers</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>18000</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Max restaurant spend</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>3000</v>
+          <t>Credit card</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Max luxury accrual</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n">
-        <v>2500</v>
-      </c>
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Cooling-off period for purchases &gt; ₹5,000</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>7 days</t>
-        </is>
-      </c>
+          <t>Living budget (from salary only)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Credit card bill cap</t>
+          <t>Restaurants + street food + snacks</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>8000</v>
-      </c>
+        <v>5600</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Transport + subscriptions</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Healthcare + shopping + misc</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Groceries from salary</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Total living from salary</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>30200</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Projected salary surplus</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>8653</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Total wealth building (Zerodha + surplus)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>128653</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Wealth rate (% of salary)</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Transfer ₹1.2L to Zerodha</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>1st–2nd of month</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Use Pluxee for all groceries first</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DMart / BigBasket</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Max restaurant spend</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cooling-off for purchases &gt; ₹5,000</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>No credit card bills</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>UPI/debit only</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>Next Month — Salary Allocation Plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Amount (₹)</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Transfer to Zerodha</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1st–2nd</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Family transfer (Somasundar etc.)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1st week</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Load Pluxee — groceries</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>5600</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Auto/credited</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Employer benefit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Restaurants (max 2 outings)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Through month</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Office lunch / street food</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Through month</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Snacks + desserts + office cafe</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Through month</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Metro transport</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Through month</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Cursor AI + subscriptions</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare / pharmacy</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Shopping (non-essential)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>As needed</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Misc / emergency buffer</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Groceries</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Use Pluxee only</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Pluxee</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>SALARY OUTFLOW TOTAL</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>150200</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PROJECTED SALARY SURPLUS</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>8653</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Keep in bank / sweep FD</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>TOTAL WEALTH BUILDING</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>128653</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Zerodha + savings</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Treat pharmacy as one-time: reduce healthcare budget to ₹200 buffer
June Sparsh Hospital (₹2,290) was one-off; projected surplus now ~₹9,953

Co-authored-by: Shivam Modnaval <ShivamModanval5268@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget-tracker/monthly_budget_tracker.xlsx
+++ b/budget-tracker/monthly_budget_tracker.xlsx
@@ -892,7 +892,7 @@
         <v>2290</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
@@ -907,7 +907,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Variable; claim via corporate insurance</t>
+          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>30200</v>
+        <v>28900</v>
       </c>
     </row>
     <row r="27">
@@ -2126,7 +2126,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>30200</v>
+        <v>28900</v>
       </c>
     </row>
     <row r="19">
@@ -2140,7 +2140,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>8653</v>
+        <v>9953</v>
       </c>
     </row>
     <row r="21">
@@ -2150,7 +2150,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>128653</v>
+        <v>129953</v>
       </c>
     </row>
     <row r="22">
@@ -2160,7 +2160,7 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>81</v>
+        <v>81.8</v>
       </c>
     </row>
     <row r="23">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>150200</v>
+        <v>148900</v>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
@@ -2590,7 +2590,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>8653</v>
+        <v>9953</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>128653</v>
+        <v>129953</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recategorize Somasundar ₹16K as monthly rent, not family transfer
- Rent is fixed ₹16,000/month on 1st
- Personal transfers (Rajat/Govind) budgeted at ₹0 unless recurring
- Projected surplus now ~₹11,953

Co-authored-by: Shivam Modnaval <ShivamModanval5268@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget-tracker/monthly_budget_tracker.xlsx
+++ b/budget-tracker/monthly_budget_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -537,14 +537,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Family transfers</t>
+          <t>Rent (Somasundar)</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>18060</v>
+        <v>16000</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>0</v>
@@ -559,18 +559,18 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Fixed obligation — budget as non-negotiable</t>
+          <t>Monthly rent — pay on 1st of month via UPI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Credit card payment</t>
+          <t>Personal transfers</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>13180</v>
+        <v>2060</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -588,21 +588,21 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No CC bills — pay everything via UPI/debit</t>
+          <t>June: Rajat ₹1,100 + Govind ₹960 — budget only if recurring</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Pluxee — groceries (benefit)</t>
+          <t>Credit card payment</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>13180</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5600</v>
+        <v>0</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>0</v>
@@ -617,21 +617,21 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>₹4,400 + ₹1,200 loaded monthly; DMart/BigBasket only</t>
+          <t>No CC bills — pay everything via UPI/debit</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Groceries (from salary)</t>
+          <t>Pluxee — groceries (benefit)</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2178</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0</v>
+        <v>5600</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>0</v>
@@ -646,21 +646,21 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Use Pluxee first; salary only if Pluxee exhausted</t>
+          <t>₹4,400 + ₹1,200 loaded monthly; DMart/BigBasket only</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Restaurant dining</t>
+          <t>Groceries (from salary)</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>5253</v>
+        <v>2178</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2500</v>
+        <v>0</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>0</v>
@@ -675,18 +675,18 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Max 2 sit-down meals per month</t>
+          <t>Use Pluxee first; salary only if Pluxee exhausted</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Street food / canteen</t>
+          <t>Restaurant dining</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>3594</v>
+        <v>5253</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>2500</v>
@@ -704,21 +704,21 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Office lunch — use Infosys cafeteria when possible</t>
+          <t>Max 2 sit-down meals per month</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Desserts (Polar Bear etc.)</t>
+          <t>Street food / canteen</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>924</v>
+        <v>3594</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>300</v>
+        <v>2500</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0</v>
@@ -733,18 +733,18 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Max 1 visit per month</t>
+          <t>Office lunch — use Infosys cafeteria when possible</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Office snacks / tea</t>
+          <t>Desserts (Polar Bear etc.)</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>750</v>
+        <v>924</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>300</v>
@@ -762,21 +762,21 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Carry flask; avoid daily ₹35 UPI</t>
+          <t>Max 1 visit per month</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Office cafe (Cowrks)</t>
+          <t>Office snacks / tea</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>598</v>
+        <v>750</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>0</v>
@@ -791,18 +791,18 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Use only when necessary</t>
+          <t>Carry flask; avoid daily ₹35 UPI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Transport (Metro)</t>
+          <t>Office cafe (Cowrks)</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>180</v>
+        <v>598</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>200</v>
@@ -820,21 +820,21 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Already optimal</t>
+          <t>Use only when necessary</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Software subscriptions</t>
+          <t>Transport (Metro)</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>2376</v>
+        <v>180</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>0</v>
@@ -849,21 +849,21 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Cursor AI — review tier / annual plan</t>
+          <t>Already optimal</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Other subscriptions</t>
+          <t>Software subscriptions</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2</v>
+        <v>2376</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -878,18 +878,18 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>YouTube, streaming, etc.</t>
+          <t>Cursor AI — review tier / annual plan</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Other subscriptions</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>2290</v>
+        <v>2</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>200</v>
@@ -907,21 +907,21 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
+          <t>YouTube, streaming, etc.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Education / training</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>1875</v>
+        <v>2290</v>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>0</v>
@@ -936,21 +936,21 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Only if actively enrolled in a course</t>
+          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Shopping (Amazon etc.)</t>
+          <t>Education / training</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1842</v>
+        <v>1875</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0</v>
@@ -965,21 +965,21 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Non-essential purchases only</t>
+          <t>Only if actively enrolled in a course</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Gift cards</t>
+          <t>Shopping (Amazon etc.)</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>4240</v>
+        <v>1842</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
@@ -994,18 +994,18 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Avoid prepaid unless planned gift</t>
+          <t>Non-essential purchases only</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Luxury / big purchases</t>
+          <t>Gift cards</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>30867</v>
+        <v>4240</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>0</v>
@@ -1023,21 +1023,21 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
+          <t>Avoid prepaid unless planned gift</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Misc / buffer</t>
+          <t>Luxury / big purchases</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0</v>
+        <v>30867</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>0</v>
@@ -1052,93 +1052,122 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
+          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Misc / buffer</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3">
+        <f>D21-C21</f>
+        <v/>
+      </c>
+      <c r="F21" s="2">
+        <f>IF(D21=0,"Enter spend",IF(E21&lt;=0,"✓ On track","⚠ Over"))</f>
+        <v/>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
           <t>Unexpected expenses from salary</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>TOTAL (excl. income)</t>
         </is>
       </c>
-      <c r="B21" s="5">
-        <f>SUM(B2:B20)</f>
-        <v/>
-      </c>
-      <c r="C21" s="5">
-        <f>SUM(C2:C20)</f>
-        <v/>
-      </c>
-      <c r="D21" s="5">
-        <f>SUM(D2:D20)</f>
-        <v/>
-      </c>
-      <c r="E21" s="5">
-        <f>D21-C21</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Monthly salary (bank)</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>158853</v>
-      </c>
-    </row>
+      <c r="B22" s="5">
+        <f>SUM(B2:B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>SUM(C2:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>SUM(D2:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>D22-C22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Pluxee grocery benefit (separate)</t>
+          <t>Monthly salary (bank)</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
-        <v>5600</v>
+        <v>158853</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Zerodha investment target</t>
+          <t>Pluxee grocery benefit (separate)</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>120000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Living spend from salary (target)</t>
+          <t>Zerodha investment target</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>28900</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Projected salary surplus (Salary − Actual spend)</t>
-        </is>
-      </c>
-      <c r="D27" s="5">
-        <f>C23-D21</f>
-        <v/>
+          <t>Living spend from salary (target)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>26900</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>Projected salary surplus (Salary − Actual spend)</t>
+        </is>
+      </c>
+      <c r="D28" s="5">
+        <f>C24-D22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
           <t>Total to Zerodha + surplus wealth</t>
         </is>
       </c>
-      <c r="C28" s="5">
-        <f>C25+C27</f>
+      <c r="C29" s="5">
+        <f>C26+C28</f>
         <v/>
       </c>
     </row>
@@ -1505,7 +1534,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Investments (Zerodha),Family transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Restaurant dining,Street food / canteen,Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
+      <formula1>"Investments (Zerodha),Rent (Somasundar),Personal transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Restaurant dining,Street food / canteen,Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Debit,Credit"</formula1>
@@ -1571,7 +1600,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Family transfers</t>
+          <t>Rent (Somasundar)</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
@@ -1846,7 +1875,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Family transfers</t>
+          <t>Personal transfers</t>
         </is>
       </c>
       <c r="D13" s="5" t="n">
@@ -1969,7 +1998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2050,184 +2079,194 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Family transfers</t>
+          <t>Rent (Somasundar)</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>18000</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>Personal transfers</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>Credit card</t>
         </is>
       </c>
-      <c r="B11" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Living budget (from salary only)</t>
-        </is>
-      </c>
+      <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Restaurants + street food + snacks</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>5600</v>
-      </c>
+          <t>Living budget (from salary only)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Transport + subscriptions</t>
+          <t>Restaurants + street food + snacks</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>1700</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Healthcare + shopping + misc</t>
+          <t>Transport + subscriptions</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>4500</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Groceries from salary</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>0</v>
+          <t>Healthcare + shopping + misc</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>3200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>Groceries from salary</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>Total living from salary</t>
         </is>
       </c>
-      <c r="B18" s="5" t="n">
-        <v>28900</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr"/>
+      <c r="B19" s="5" t="n">
+        <v>26900</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Projected salary surplus</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>9953</v>
-      </c>
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Total wealth building (Zerodha + surplus)</t>
+          <t>Projected salary surplus</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>129953</v>
+        <v>11953</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Total wealth building (Zerodha + surplus)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>131953</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Wealth rate (% of salary)</t>
         </is>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>81.8</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr"/>
-      <c r="B23" t="inlineStr"/>
+      <c r="B23" s="7" t="n">
+        <v>83.09999999999999</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Rules</t>
-        </is>
-      </c>
+      <c r="A24" t="inlineStr"/>
       <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Transfer ₹1.2L to Zerodha</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1st–2nd of month</t>
-        </is>
-      </c>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Use Pluxee for all groceries first</t>
+          <t>Transfer ₹1.2L to Zerodha</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>DMart / BigBasket</t>
+          <t>1st–2nd of month</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Max restaurant spend</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="n">
-        <v>2500</v>
+          <t>Use Pluxee for all groceries first</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DMart / BigBasket</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cooling-off for purchases &gt; ₹5,000</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>7 days</t>
-        </is>
+          <t>Max restaurant spend</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>2500</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>Cooling-off for purchases &gt; ₹5,000</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>No credit card bills</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>UPI/debit only</t>
         </is>
@@ -2248,9 +2287,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -2318,15 +2357,15 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Family transfer (Somasundar etc.)</t>
+          <t>Rent — Somasundar</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>18000</v>
+        <v>16000</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>1st week</t>
+          <t>1st of month</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2479,15 +2518,15 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Healthcare / pharmacy</t>
+          <t>Healthcare / pharmacy (buffer only)</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>As needed</t>
+          <t>As needed — June was one-time</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2573,7 +2612,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>148900</v>
+        <v>146900</v>
       </c>
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
@@ -2590,7 +2629,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>9953</v>
+        <v>11953</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -2611,7 +2650,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>129953</v>
+        <v>131953</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add ₹2,000/month weekend expense envelope (₹500 per weekend)
- Weekends: dining, outings, leisure capped at ₹2K
- Weekday restaurants reduced to ₹500; Rajat/Govind confirmed one-time

Co-authored-by: Shivam Modnaval <ShivamModanval5268@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget-tracker/monthly_budget_tracker.xlsx
+++ b/budget-tracker/monthly_budget_tracker.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -682,14 +682,14 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Restaurant dining</t>
+          <t>Weekend expenses</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>5253</v>
+        <v>0</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>0</v>
@@ -704,21 +704,21 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Max 2 sit-down meals per month</t>
+          <t>Sat–Sun only: dining, outings, leisure — ₹500 per weekend</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Street food / canteen</t>
+          <t>Restaurant dining (weekdays)</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3594</v>
+        <v>5253</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0</v>
@@ -733,21 +733,21 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Office lunch — use Infosys cafeteria when possible</t>
+          <t>Rare weekday sit-down; weekends use weekend envelope</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Desserts (Polar Bear etc.)</t>
+          <t>Street food / canteen (weekdays)</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>924</v>
+        <v>3594</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>300</v>
+        <v>2500</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>0</v>
@@ -762,18 +762,18 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Max 1 visit per month</t>
+          <t>Mon–Fri office lunch — use Infosys cafeteria</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Office snacks / tea</t>
+          <t>Desserts (Polar Bear etc.)</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>750</v>
+        <v>924</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>300</v>
@@ -791,21 +791,21 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Carry flask; avoid daily ₹35 UPI</t>
+          <t>Max 1 visit per month</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Office cafe (Cowrks)</t>
+          <t>Office snacks / tea</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>598</v>
+        <v>750</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>0</v>
@@ -820,18 +820,18 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Use only when necessary</t>
+          <t>Carry flask; avoid daily ₹35 UPI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Transport (Metro)</t>
+          <t>Office cafe (Cowrks)</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>180</v>
+        <v>598</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>200</v>
@@ -849,21 +849,21 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Already optimal</t>
+          <t>Use only when necessary</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Software subscriptions</t>
+          <t>Transport (Metro)</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>2376</v>
+        <v>180</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>0</v>
@@ -878,21 +878,21 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Cursor AI — review tier / annual plan</t>
+          <t>Already optimal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Other subscriptions</t>
+          <t>Software subscriptions</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>2</v>
+        <v>2376</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>200</v>
+        <v>1500</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>0</v>
@@ -907,18 +907,18 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>YouTube, streaming, etc.</t>
+          <t>Cursor AI — review tier / annual plan</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Other subscriptions</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>2290</v>
+        <v>2</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>200</v>
@@ -936,21 +936,21 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
+          <t>YouTube, streaming, etc.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Education / training</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>1875</v>
+        <v>2290</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0</v>
@@ -965,21 +965,21 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Only if actively enrolled in a course</t>
+          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Shopping (Amazon etc.)</t>
+          <t>Education / training</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>1842</v>
+        <v>1875</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
@@ -994,21 +994,21 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Non-essential purchases only</t>
+          <t>Only if actively enrolled in a course</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Gift cards</t>
+          <t>Shopping (Amazon etc.)</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>4240</v>
+        <v>1842</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0</v>
@@ -1023,18 +1023,18 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Avoid prepaid unless planned gift</t>
+          <t>Non-essential purchases only</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Luxury / big purchases</t>
+          <t>Gift cards</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>30867</v>
+        <v>4240</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>0</v>
@@ -1052,21 +1052,21 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
+          <t>Avoid prepaid unless planned gift</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Misc / buffer</t>
+          <t>Luxury / big purchases</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0</v>
+        <v>30867</v>
       </c>
       <c r="C21" s="3" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
@@ -1081,93 +1081,122 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
+          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Misc / buffer</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <f>D22-C22</f>
+        <v/>
+      </c>
+      <c r="F22" s="2">
+        <f>IF(D22=0,"Enter spend",IF(E22&lt;=0,"✓ On track","⚠ Over"))</f>
+        <v/>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
           <t>Unexpected expenses from salary</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>TOTAL (excl. income)</t>
         </is>
       </c>
-      <c r="B22" s="5">
-        <f>SUM(B2:B21)</f>
-        <v/>
-      </c>
-      <c r="C22" s="5">
-        <f>SUM(C2:C21)</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>SUM(D2:D21)</f>
-        <v/>
-      </c>
-      <c r="E22" s="5">
-        <f>D22-C22</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23"/>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Monthly salary (bank)</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>158853</v>
-      </c>
-    </row>
+      <c r="B23" s="5">
+        <f>SUM(B2:B22)</f>
+        <v/>
+      </c>
+      <c r="C23" s="5">
+        <f>SUM(C2:C22)</f>
+        <v/>
+      </c>
+      <c r="D23" s="5">
+        <f>SUM(D2:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="5">
+        <f>D23-C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Pluxee grocery benefit (separate)</t>
+          <t>Monthly salary (bank)</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
-        <v>5600</v>
+        <v>158853</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Zerodha investment target</t>
+          <t>Pluxee grocery benefit (separate)</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
-        <v>120000</v>
+        <v>5600</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Living spend from salary (target)</t>
+          <t>Zerodha investment target</t>
         </is>
       </c>
       <c r="C27" s="5" t="n">
-        <v>26900</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Projected salary surplus (Salary − Actual spend)</t>
-        </is>
-      </c>
-      <c r="D28" s="5">
-        <f>C24-D22</f>
-        <v/>
+          <t>Living spend from salary (target)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>26900</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>Projected salary surplus (Salary − Actual spend)</t>
+        </is>
+      </c>
+      <c r="D29" s="5">
+        <f>C25-D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
           <t>Total to Zerodha + surplus wealth</t>
         </is>
       </c>
-      <c r="C29" s="5">
-        <f>C26+C28</f>
+      <c r="C30" s="5">
+        <f>C27+C29</f>
         <v/>
       </c>
     </row>
@@ -1534,7 +1563,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Investments (Zerodha),Rent (Somasundar),Personal transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Restaurant dining,Street food / canteen,Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
+      <formula1>"Investments (Zerodha),Rent (Somasundar),Personal transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Weekend expenses,Restaurant dining (weekdays),Street food / canteen (weekdays),Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Debit,Credit"</formula1>

</xml_diff>

<commit_message>
Sanitize budget-tracker: remove PII from public repo files
- Replace real names, UPI handles, employer, and exact salary with generics
- Add config.py defaults + local_config.example.py for private local values
- Gitignore local_config.py and user bank CSV exports
- Generic sample_statement.csv and sample baseline in Excel workbook

Co-authored-by: hacktrash7 <hacktrash7@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/budget-tracker/monthly_budget_tracker.xlsx
+++ b/budget-tracker/monthly_budget_tracker.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Budget vs Actual" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Transaction Log" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="June 2026 Baseline" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sample Baseline" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Dashboard" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Monthly Plan" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
@@ -460,7 +460,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -476,7 +476,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>June Actual (₹)</t>
+          <t>Sample Actual (₹)</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>71000</v>
+        <v>65000</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>120000</v>
@@ -530,18 +530,18 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Transfer ₹1.2L to Zerodha on 1st–2nd of month</t>
+          <t>Transfer to Zerodha on 1st–2nd of month</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Rent (Somasundar)</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>16000</v>
+        <v>15000</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>16000</v>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>2060</v>
+        <v>1000</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -588,7 +588,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>June: Rajat ₹1,100 + Govind ₹960 — budget only if recurring</t>
+          <t>Budget only for recurring transfers</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>13180</v>
+        <v>10000</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0</v>
@@ -646,7 +646,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>₹4,400 + ₹1,200 loaded monthly; DMart/BigBasket only</t>
+          <t>Corporate meal/grocery benefit; supermarket only</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2178</v>
+        <v>2000</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0</v>
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>5253</v>
+        <v>4000</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>500</v>
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>3594</v>
+        <v>3000</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>2500</v>
@@ -762,18 +762,18 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Mon–Fri office lunch — use Infosys cafeteria</t>
+          <t>Mon–Fri office lunch — use office cafeteria</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Desserts (Polar Bear etc.)</t>
+          <t>Desserts</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>924</v>
+        <v>800</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>300</v>
@@ -802,7 +802,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>750</v>
+        <v>600</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>300</v>
@@ -820,18 +820,18 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Carry flask; avoid daily ₹35 UPI</t>
+          <t>Carry flask; avoid daily small UPI payments</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Office cafe (Cowrks)</t>
+          <t>Office cafe</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>598</v>
+        <v>500</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>200</v>
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>200</v>
@@ -878,7 +878,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Already optimal</t>
+          <t>Commute</t>
         </is>
       </c>
     </row>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>2376</v>
+        <v>1500</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>1500</v>
@@ -907,7 +907,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Cursor AI — review tier / annual plan</t>
+          <t>Dev tools / subscriptions — review tier annually</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>200</v>
@@ -936,7 +936,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>YouTube, streaming, etc.</t>
+          <t>Streaming, etc.</t>
         </is>
       </c>
     </row>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>2290</v>
+        <v>2000</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>200</v>
@@ -965,7 +965,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>One-time in June (Sparsh Hospital); keep small buffer only</t>
+          <t>Buffer only unless recurring medical need</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>1875</v>
+        <v>1500</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0</v>
@@ -1001,11 +1001,11 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Shopping (Amazon etc.)</t>
+          <t>Shopping (online)</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>1842</v>
+        <v>1500</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>1000</v>
@@ -1034,7 +1034,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>4240</v>
+        <v>2000</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>0</v>
@@ -1063,7 +1063,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>30867</v>
+        <v>5000</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>0</v>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>No luxury spend — use 7-day rule if &gt; ₹5,000</t>
+          <t>No unplanned luxury — 7-day rule if &gt; ₹5,000</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1563,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Investments (Zerodha),Rent (Somasundar),Personal transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Weekend expenses,Restaurant dining (weekdays),Street food / canteen (weekdays),Desserts (Polar Bear etc.),Office snacks / tea,Office cafe (Cowrks),Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (Amazon etc.),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
+      <formula1>"Investments (Zerodha),Rent,Personal transfers,Credit card payment,Pluxee — groceries (benefit),Groceries (from salary),Weekend expenses,Restaurant dining (weekdays),Street food / canteen (weekdays),Desserts,Office snacks / tea,Office cafe,Transport (Metro),Software subscriptions,Other subscriptions,Healthcare,Education / training,Shopping (online),Gift cards,Luxury / big purchases,Misc / buffer,Income,Pluxee — groceries (benefit),Misc / buffer"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Debit,Credit"</formula1>
@@ -1579,12 +1579,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1624,12 +1624,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SOMASUNDAR</t>
+          <t>Landlord — rent</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Rent (Somasundar)</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="D2" s="5" t="n">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sparsh Hospital</t>
+          <t>City Hospital</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>2290</v>
+        <v>2000</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>71000</v>
+        <v>65000</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>13180</v>
+        <v>10000</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1719,21 +1719,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>01-Jun</t>
+          <t>03-Jun</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Centre for</t>
+          <t>Supermarket</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Education / training</t>
+          <t>Groceries</t>
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>1875</v>
+        <v>900</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1744,21 +1744,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03-Jun</t>
+          <t>07-Jun</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DMart</t>
+          <t>Restaurant</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Groceries</t>
+          <t>Restaurant dining (weekdays)</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>911</v>
+        <v>800</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1769,21 +1769,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07-Jun</t>
+          <t>15-Jun</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Munchzeste</t>
+          <t>Software subscription</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Restaurant dining</t>
+          <t>Software subscriptions</t>
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>1125</v>
+        <v>1500</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1794,21 +1794,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>10-Jun</t>
+          <t>17-Jun</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TR Enterprise</t>
+          <t>Online store</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Restaurant dining</t>
+          <t>Shopping (online)</t>
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>1070</v>
+        <v>1000</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1819,21 +1819,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>15-Jun</t>
+          <t>28-Jun</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cursor AI</t>
+          <t>Retail store</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Software subscriptions</t>
+          <t>Luxury / big purchases</t>
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>2376</v>
+        <v>5000</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1844,173 +1844,23 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>17-Jun</t>
+          <t>30-Jun</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Amazon gift card</t>
+          <t>Salary — Employer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Gift cards</t>
+          <t>Income</t>
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>4240</v>
+        <v>158853</v>
       </c>
       <c r="E11" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>21-Jun</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Chulha Cha</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Restaurant dining</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>1180</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>21-Jun</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Rajat Agarwal</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Personal transfers</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>1100</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>28-Jun</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Titan</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Luxury / big purchases</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>30867</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>28-Jun</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Truffles</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Restaurant dining</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>1155</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>28-Jun</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>FGM</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Shopping (Amazon etc.)</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>1502</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Debit</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>30-Jun</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Salary — Johnson Controls</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>158853</v>
-      </c>
-      <c r="E17" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
@@ -2027,17 +1877,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Monthly Budget Dashboard — Updated Plan</t>
+          <t>Monthly Budget Dashboard</t>
         </is>
       </c>
     </row>
@@ -2066,7 +1916,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Pluxee groceries (₹4,400 + ₹1,200)</t>
+          <t>Pluxee groceries</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
@@ -2108,7 +1958,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Rent (Somasundar)</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
@@ -2150,152 +2000,162 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Restaurants + street food + snacks</t>
+          <t>Weekday food + snacks</t>
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>5600</v>
+        <v>3300</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Transport + subscriptions</t>
+          <t>Weekend expenses (Sat–Sun)</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>1700</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Healthcare + shopping + misc</t>
+          <t>Transport + subscriptions</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>3200</v>
+        <v>1700</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Groceries from salary</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0</v>
+          <t>Healthcare + shopping + misc</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>3200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>Groceries from salary</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Total living from salary</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B20" s="5" t="n">
         <v>26900</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Projected salary surplus</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="n">
-        <v>11953</v>
-      </c>
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Total wealth building (Zerodha + surplus)</t>
+          <t>Projected salary surplus</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>131953</v>
+        <v>11953</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Total wealth building (Zerodha + surplus)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>131953</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Wealth rate (% of salary)</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n">
+      <c r="B24" s="7" t="n">
         <v>83.09999999999999</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-      <c r="B24" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Rules</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
       <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Transfer ₹1.2L to Zerodha</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1st–2nd of month</t>
-        </is>
-      </c>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Use Pluxee for all groceries first</t>
+          <t>Transfer to Zerodha</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>DMart / BigBasket</t>
+          <t>1st–2nd of month</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Max restaurant spend</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="n">
-        <v>2500</v>
+          <t>Use Pluxee for groceries first</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Supermarket</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cooling-off for purchases &gt; ₹5,000</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>7 days</t>
-        </is>
+          <t>Weekend cap</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Cooling-off for purchases &gt; ₹5,000</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>7 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>No credit card bills</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>UPI/debit only</t>
         </is>
@@ -2312,20 +2172,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Next Month — Salary Allocation Plan</t>
+          <t>Monthly Salary Allocation Plan</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2246,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Rent — Somasundar</t>
+          <t>Rent</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -2409,7 +2269,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Load Pluxee — groceries</t>
+          <t>Pluxee — groceries</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
@@ -2432,15 +2292,15 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Restaurants (max 2 outings)</t>
+          <t>Weekend expenses (Sat–Sun)</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2500</v>
+        <v>2000</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Through month</t>
+          <t>₹500 per weekend × 4</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -2455,15 +2315,15 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Office lunch / street food</t>
+          <t>Weekday restaurants (optional)</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2500</v>
+        <v>500</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Through month</t>
+          <t>Mon–Fri only</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -2478,11 +2338,11 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Snacks + desserts + office cafe</t>
+          <t>Office lunch / street food (Mon–Fri)</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>500</v>
+        <v>2500</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -2501,15 +2361,15 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Metro transport</t>
+          <t>Snacks + desserts + office cafe</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Through month</t>
+          <t>Mon–Fri</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -2524,15 +2384,15 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Cursor AI + subscriptions</t>
+          <t>Metro transport</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1700</v>
+        <v>200</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Monthly</t>
+          <t>Through month</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -2547,15 +2407,15 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Healthcare / pharmacy (buffer only)</t>
+          <t>Software + subscriptions</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>200</v>
+        <v>1700</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>As needed — June was one-time</t>
+          <t>Monthly</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -2570,11 +2430,11 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Shopping (non-essential)</t>
+          <t>Healthcare buffer</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -2593,15 +2453,15 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Misc / emergency buffer</t>
+          <t>Shopping (non-essential)</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>As needed</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -2616,37 +2476,43 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>Misc / emergency buffer</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Reserve</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>Groceries</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="C16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Use Pluxee only</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Pluxee</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>SALARY OUTFLOW TOTAL</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="n">
-        <v>146900</v>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Salary</t>
         </is>
       </c>
     </row>
@@ -2654,17 +2520,13 @@
       <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PROJECTED SALARY SURPLUS</t>
+          <t>SALARY OUTFLOW TOTAL</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>11953</v>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Keep in bank / sweep FD</t>
-        </is>
-      </c>
+        <v>146900</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Salary</t>
@@ -2675,18 +2537,39 @@
       <c r="A18" s="2" t="inlineStr"/>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t>PROJECTED SALARY SURPLUS</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>11953</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Keep in bank / sweep FD</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Salary</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
           <t>TOTAL WEALTH BUILDING</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C19" s="3" t="n">
         <v>131953</v>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Zerodha + savings</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>